<commit_message>
Fix 1325 Missing Columns
</commit_message>
<xml_diff>
--- a/TaxMaster.Infra/Assets/1325Form.xlsx
+++ b/TaxMaster.Infra/Assets/1325Form.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ybenharosh\source\repos\TaxMaster\TaxMaster.Infra\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C06F160-1969-42FC-B625-7FA8BED44A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21033FED-5E15-41BE-8C15-102F616C863D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2EAC2B80-7C28-4C96-B290-8BE40F8543A1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2EAC2B80-7C28-4C96-B290-8BE40F8543A1}"/>
   </bookViews>
   <sheets>
     <sheet name="1325" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'1325'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'1325'!$A$1:$M$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>חתימה</t>
   </si>
@@ -83,12 +83,15 @@
     <t>כן</t>
   </si>
   <si>
+    <t>:תיק מספר</t>
+  </si>
+  <si>
+    <t>חותמת המייצג לשם זיהוי</t>
+  </si>
+  <si>
     <t>:הנישום שם</t>
   </si>
   <si>
-    <t>:תיק מספר</t>
-  </si>
-  <si>
     <t>:ל"בחו נכס</t>
   </si>
   <si>
@@ -96,6 +99,12 @@
   </si>
   <si>
     <t>מכירות סכום</t>
+  </si>
+  <si>
+    <t>המס לשנת סחירים ערך מניירות הון רווח</t>
+  </si>
+  <si>
+    <t>השנתי הדוח לטופס ג(1) נספח</t>
   </si>
 </sst>
 </file>
@@ -109,7 +118,7 @@
     <numFmt numFmtId="166" formatCode="[$-1010000]d/m/yyyy;@"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +135,14 @@
       <charset val="177"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="36"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -135,7 +152,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -147,96 +164,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -381,101 +308,200 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1014,8 +1040,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{331D903F-145D-4022-9AB6-9A1FC3AD8457}" name="Table53" displayName="Table53" ref="A4:L24" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
-  <autoFilter ref="A4:L24" xr:uid="{EDDFF828-E11C-4C14-974A-F5FB5050A084}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{331D903F-145D-4022-9AB6-9A1FC3AD8457}" name="Table53" displayName="Table53" ref="A6:L26" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+  <autoFilter ref="A6:L26" xr:uid="{EDDFF828-E11C-4C14-974A-F5FB5050A084}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{10D4D436-818E-4F8E-ACBF-6A12B900601E}" name=" " dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{2F9CBED6-E433-43FA-A017-97779ABA6D45}" name="זיהוי מלא של נייר הערך שנמכר לפי הסדר הכרונולוגי של המכירות" dataDxfId="10"/>
@@ -1351,7 +1377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C952D2-02CC-494D-825B-79121DB2144F}">
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="20.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.125" style="1" bestFit="1" customWidth="1"/>
@@ -1363,426 +1389,452 @@
     <col min="7" max="7" width="16.5" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5" style="1" customWidth="1"/>
     <col min="11" max="11" width="20.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.5" style="1" customWidth="1"/>
     <col min="13" max="16384" width="8" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D2" s="29" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="C2" s="32"/>
+      <c r="D2" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="28"/>
-      <c r="F2" s="29" t="s">
+      <c r="G4" s="33"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" s="11" customFormat="1" ht="98.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="L6" s="19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="18">
+        <v>1</v>
+      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="12"/>
+    </row>
+    <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="18">
+        <v>2</v>
+      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="12"/>
+    </row>
+    <row r="9" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="18">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="12"/>
+    </row>
+    <row r="10" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="18">
+        <v>4</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="12"/>
+    </row>
+    <row r="11" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="18">
+        <v>5</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="12"/>
+    </row>
+    <row r="12" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="18">
+        <v>6</v>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="12"/>
+    </row>
+    <row r="13" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="18">
+        <v>7</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="12"/>
+    </row>
+    <row r="14" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="18">
+        <v>8</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="12"/>
+    </row>
+    <row r="15" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="18">
+        <v>9</v>
+      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="12"/>
+    </row>
+    <row r="16" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="18">
+        <v>10</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="12"/>
+    </row>
+    <row r="17" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="18">
+        <v>11</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="12"/>
+    </row>
+    <row r="18" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="18">
+        <v>12</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="12"/>
+    </row>
+    <row r="19" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="18">
+        <v>13</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="12"/>
+    </row>
+    <row r="20" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="18">
+        <v>14</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="12"/>
+    </row>
+    <row r="21" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="18">
         <v>15</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="29" t="s">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="12"/>
+    </row>
+    <row r="22" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="18">
         <v>16</v>
       </c>
-      <c r="J2" s="28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" s="13" customFormat="1" ht="98.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="J4" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="K4" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="L4" s="21" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="20">
-        <v>1</v>
-      </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="14"/>
-    </row>
-    <row r="6" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="20">
-        <v>2</v>
-      </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="14"/>
-    </row>
-    <row r="7" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20">
-        <v>3</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="14"/>
-    </row>
-    <row r="8" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="20">
-        <v>4</v>
-      </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="14"/>
-    </row>
-    <row r="9" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="20">
-        <v>5</v>
-      </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="14"/>
-    </row>
-    <row r="10" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20">
-        <v>6</v>
-      </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="14"/>
-    </row>
-    <row r="11" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="20">
-        <v>7</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="14"/>
-    </row>
-    <row r="12" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="20">
-        <v>8</v>
-      </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="14"/>
-    </row>
-    <row r="13" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20">
-        <v>9</v>
-      </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="14"/>
-    </row>
-    <row r="14" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="20">
-        <v>10</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="14"/>
-    </row>
-    <row r="15" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="20">
-        <v>11</v>
-      </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="14"/>
-    </row>
-    <row r="16" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="20">
-        <v>12</v>
-      </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="14"/>
-    </row>
-    <row r="17" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="20">
-        <v>13</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="14"/>
-    </row>
-    <row r="18" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="20">
-        <v>14</v>
-      </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="14"/>
-    </row>
-    <row r="19" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="20">
-        <v>15</v>
-      </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="14"/>
-    </row>
-    <row r="20" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="20">
-        <v>16</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="14"/>
-    </row>
-    <row r="21" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="20">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="12"/>
+    </row>
+    <row r="23" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="18">
         <v>17</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="14"/>
-    </row>
-    <row r="22" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="12"/>
+    </row>
+    <row r="24" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="18">
         <v>18</v>
       </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="14"/>
-    </row>
-    <row r="23" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="20">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="12"/>
+    </row>
+    <row r="25" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="18">
         <v>19</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="14"/>
-    </row>
-    <row r="24" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="12">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="12"/>
+    </row>
+    <row r="26" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10">
         <v>20</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="6"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D26" s="3"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="4"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D27" s="3"/>
-      <c r="I27" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="J27" s="33"/>
-      <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D28" s="3"/>
-      <c r="I28" s="34" t="s">
+    </row>
+    <row r="29" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D29" s="3"/>
+      <c r="I29" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="J28" s="35"/>
-      <c r="K28" s="4"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D29" s="3"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="I32" s="1" t="s">
+      <c r="J29" s="39"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="28"/>
+    </row>
+    <row r="30" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D30" s="3"/>
+      <c r="I30" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="J30" s="37"/>
+      <c r="K30" s="29"/>
+      <c r="L30" s="26"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D31" s="3"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+    </row>
+    <row r="33" spans="9:12" ht="21" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="34" spans="9:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I34" s="27" t="s">
         <v>0</v>
       </c>
+      <c r="J34" s="27"/>
+      <c r="K34" s="30"/>
+      <c r="L34" s="26"/>
+    </row>
+    <row r="35" spans="9:12" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I35" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" s="30"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J30"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="58" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
re-format 1325 xl form
</commit_message>
<xml_diff>
--- a/TaxMaster.Infra/Assets/1325Form.xlsx
+++ b/TaxMaster.Infra/Assets/1325Form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ybenharosh\source\repos\TaxMaster\TaxMaster.Infra\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21033FED-5E15-41BE-8C15-102F616C863D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A475D1B-5725-493A-BFDB-EE3B46717C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2EAC2B80-7C28-4C96-B290-8BE40F8543A1}"/>
   </bookViews>
@@ -405,26 +405,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -434,21 +425,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -478,8 +460,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -491,18 +471,47 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -523,99 +532,21 @@
         <charset val="177"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="177"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="177"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -634,7 +565,7 @@
       </font>
       <numFmt numFmtId="166" formatCode="[$-1010000]d/m/yyyy;@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -647,12 +578,36 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="177"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -670,8 +625,8 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -684,12 +639,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -708,7 +657,7 @@
       </font>
       <numFmt numFmtId="167" formatCode="0.000"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -721,12 +670,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -744,8 +687,8 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -758,12 +701,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -782,7 +719,7 @@
       </font>
       <numFmt numFmtId="166" formatCode="[$-1010000]d/m/yyyy;@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -795,12 +732,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -817,27 +748,19 @@
         <charset val="177"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -854,8 +777,9 @@
         <charset val="177"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -868,12 +792,37 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="177"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="&quot;₪&quot;\ #,##0.00"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1045,16 +994,16 @@
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{10D4D436-818E-4F8E-ACBF-6A12B900601E}" name=" " dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{2F9CBED6-E433-43FA-A017-97779ABA6D45}" name="זיהוי מלא של נייר הערך שנמכר לפי הסדר הכרונולוגי של המכירות" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F9FA4B68-1BF5-430D-B865-92E3F1F141AB}" name="נרכש טרם הרישום למסחר" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{C8978294-3EC5-48B3-B5FF-F2D8063F098C}" name="ערך נקוב במכירה" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{34CEA42C-D2D8-4D6B-8140-70382AF6BFED}" name="תאריך הרכישה" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{0759BC3D-C2CF-40D0-B2C2-BCE91AAD5E06}" name="מחיר מקורי" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{8C94152A-81A3-4C3B-A256-81EDAC0DB6EB}" name="1+ שיעור עליית המדד" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{79EF7DBA-2F92-428B-9AAC-963976F158FD}" name="מחיר מתואם" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{22E44F69-D524-4B40-9AD5-04A62C329879}" name="תאריך המכירה" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{8A9645E6-D5D6-41BC-86E3-1F04B3919C7F}" name="תמורה" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{565415DF-9E1C-4FB7-8022-7ED15CD3AE1A}" name="רווח הון ריאלי בשיעור מס של 25%" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{755E733A-E3C2-41F8-9B51-9FD17B6D5D21}" name="הפסד הון" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{F9FA4B68-1BF5-430D-B865-92E3F1F141AB}" name="נרכש טרם הרישום למסחר" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C8978294-3EC5-48B3-B5FF-F2D8063F098C}" name="ערך נקוב במכירה" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{34CEA42C-D2D8-4D6B-8140-70382AF6BFED}" name="תאריך הרכישה" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{0759BC3D-C2CF-40D0-B2C2-BCE91AAD5E06}" name="מחיר מקורי" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{8C94152A-81A3-4C3B-A256-81EDAC0DB6EB}" name="1+ שיעור עליית המדד" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{79EF7DBA-2F92-428B-9AAC-963976F158FD}" name="מחיר מתואם" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{22E44F69-D524-4B40-9AD5-04A62C329879}" name="תאריך המכירה" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{8A9645E6-D5D6-41BC-86E3-1F04B3919C7F}" name="תמורה" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{565415DF-9E1C-4FB7-8022-7ED15CD3AE1A}" name="רווח הון ריאלי בשיעור מס של 25%" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{755E733A-E3C2-41F8-9B51-9FD17B6D5D21}" name="הפסד הון" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1401,387 +1350,387 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="C2" s="32"/>
-      <c r="D2" s="32" t="s">
+      <c r="C2" s="24"/>
+      <c r="D2" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="32"/>
+      <c r="E2" s="24"/>
     </row>
     <row r="3" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="26"/>
-      <c r="F4" s="27" t="s">
+      <c r="E4" s="20"/>
+      <c r="F4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="27" t="s">
+      <c r="G4" s="25"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="26" t="s">
+      <c r="J4" s="20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="11" customFormat="1" ht="98.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
+    <row r="6" spans="1:12" s="8" customFormat="1" ht="98.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18">
+    <row r="7" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
         <v>1</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="34"/>
+    </row>
+    <row r="8" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
         <v>2</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="12"/>
-    </row>
-    <row r="9" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="34"/>
+    </row>
+    <row r="9" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
         <v>3</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="12"/>
-    </row>
-    <row r="10" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="18">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="34"/>
+    </row>
+    <row r="10" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12">
         <v>4</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="12"/>
-    </row>
-    <row r="11" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="18">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="34"/>
+    </row>
+    <row r="11" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12">
         <v>5</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="12"/>
-    </row>
-    <row r="12" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="18">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="34"/>
+    </row>
+    <row r="12" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="12">
         <v>6</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="12"/>
-    </row>
-    <row r="13" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="18">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="34"/>
+    </row>
+    <row r="13" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12">
         <v>7</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="12"/>
-    </row>
-    <row r="14" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18">
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="33"/>
+      <c r="K13" s="33"/>
+      <c r="L13" s="34"/>
+    </row>
+    <row r="14" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12">
         <v>8</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="12"/>
-    </row>
-    <row r="15" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="18">
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="33"/>
+      <c r="L14" s="34"/>
+    </row>
+    <row r="15" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12">
         <v>9</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="12"/>
-    </row>
-    <row r="16" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="18">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="34"/>
+    </row>
+    <row r="16" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="12">
         <v>10</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="12"/>
-    </row>
-    <row r="17" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="18">
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="34"/>
+    </row>
+    <row r="17" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="12">
         <v>11</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="12"/>
-    </row>
-    <row r="18" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="18">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="34"/>
+    </row>
+    <row r="18" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12">
         <v>12</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="12"/>
-    </row>
-    <row r="19" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="18">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="34"/>
+    </row>
+    <row r="19" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12">
         <v>13</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="12"/>
-    </row>
-    <row r="20" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="18">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="34"/>
+    </row>
+    <row r="20" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="12">
         <v>14</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="12"/>
-    </row>
-    <row r="21" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="18">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="34"/>
+    </row>
+    <row r="21" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="12">
         <v>15</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="12"/>
-    </row>
-    <row r="22" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="18">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="34"/>
+    </row>
+    <row r="22" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="12">
         <v>16</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="12"/>
-    </row>
-    <row r="23" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="34"/>
+    </row>
+    <row r="23" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="12">
         <v>17</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="12"/>
-    </row>
-    <row r="24" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="18">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="33"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="34"/>
+    </row>
+    <row r="24" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="12">
         <v>18</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="12"/>
-    </row>
-    <row r="25" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="18">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="34"/>
+    </row>
+    <row r="25" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="12">
         <v>19</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="12"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10">
+      <c r="A26" s="7">
         <v>20</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="4"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="35"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="35"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="35"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="36"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D27" s="3"/>
@@ -1791,21 +1740,21 @@
     </row>
     <row r="29" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D29" s="3"/>
-      <c r="I29" s="38" t="s">
+      <c r="I29" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="J29" s="39"/>
-      <c r="K29" s="35"/>
-      <c r="L29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="39"/>
+      <c r="L29" s="40"/>
     </row>
     <row r="30" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D30" s="3"/>
-      <c r="I30" s="36" t="s">
+      <c r="I30" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="J30" s="37"/>
-      <c r="K30" s="29"/>
-      <c r="L30" s="26"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="32"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D31" s="3"/>
@@ -1815,26 +1764,27 @@
     </row>
     <row r="33" spans="9:12" ht="21" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="34" spans="9:12" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I34" s="27" t="s">
+      <c r="I34" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="J34" s="27"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="26"/>
+      <c r="J34" s="21"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="20"/>
     </row>
     <row r="35" spans="9:12" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I35" s="31" t="s">
+      <c r="I35" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="J35" s="30"/>
-      <c r="K35" s="30"/>
-      <c r="L35" s="26"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I29:J29"/>
     <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="58" orientation="landscape" r:id="rId1"/>

</xml_diff>